<commit_message>
QLDA: fix export/import/print cho danh sách dự án, KH hạng mục và phiếu trình - Export danh sách dự án: đồng bộ grid, bỏ cột ngày bắt đầu, lookup UserPortalId, regen template LetterheadExport - Import KH triển khai hạng mục: lưu CanBoChuTriId/CanBoPhoiHopIds theo UserPortalId (khớp UI combobox) - In phiếu trình KH hạng mục: format ngày Bắt đầu/Kết thúc dd/MM/yyyy - Thêm unit/integration tests và docs issues tương ứng
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/ExportTemplates/DanhSachDuAn.xlsx
+++ b/QLDA.WebApi/ExportTemplates/DanhSachDuAn.xlsx
@@ -1,22 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\ExportTemplates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2899C387-4EBA-4BAE-B136-A4007A6A3D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Data" sheetId="2" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <si>
-    <t>Trung tâm chuyển đổi số Tp Hồ Chí Minh</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
+  </si>
+  <si>
+    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc
+---------------</t>
   </si>
   <si>
     <t>DANH SÁCH DỰ ÁN</t>
@@ -34,9 +46,6 @@
     <t>Thời gian khởi công</t>
   </si>
   <si>
-    <t>Ngày bắt đầu</t>
-  </si>
-  <si>
     <t>Lãnh đạo phụ trách</t>
   </si>
   <si>
@@ -65,9 +74,6 @@
   </si>
   <si>
     <t>$thoiGianKhoiCong</t>
-  </si>
-  <si>
-    <t>$ngayBatDau</t>
   </si>
   <si>
     <t>$lanhDaoPhuTrachId</t>
@@ -91,21 +97,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="0" formatCode=""/>
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -113,7 +113,6 @@
     </font>
     <font>
       <b/>
-      <vertAlign val="baseline"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -121,7 +120,6 @@
     </font>
     <font>
       <b/>
-      <vertAlign val="baseline"/>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -137,29 +135,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC8C8C8"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="0" diagonalDown="0">
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal style="none">
-        <color rgb="FF000000"/>
-      </diagonal>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
-    <border diagonalUp="0" diagonalDown="0">
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -172,83 +160,55 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal style="none">
-        <color rgb="FF000000"/>
-      </diagonal>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="1" hidden="0"/>
-    </xf>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="1" hidden="0"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -536,97 +496,107 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="12" max="16384" width="9.140625" style="1" customWidth="1"/>
-    <col min="1" max="1" width="6.710625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.710625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.710625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.710625" style="1" customWidth="1"/>
-    <col min="5" max="6" width="30.710625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="28.710625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="25.710625" style="1" customWidth="1"/>
-    <col min="9" max="10" width="22.710625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="26.710625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="42.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="3" customWidth="1"/>
+    <col min="6" max="7" width="22.6640625" style="3" customWidth="1"/>
+    <col min="8" max="9" width="20.6640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="24" customHeight="1">
+    <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:11">
-      <c r="C3" s="3"/>
-      <c r="H3" s="3"/>
+    <row r="3" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="G4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="J4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K4" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="8" t="s">
+    <row r="5" spans="1:10" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="8" t="s">
@@ -638,29 +608,22 @@
       <c r="G5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="8" t="s">
         <v>20</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="F1:J2"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <headerFooter/>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>